<commit_message>
Migração para API concluída com sucesso
</commit_message>
<xml_diff>
--- a/DadosClima/clima.xlsx
+++ b/DadosClima/clima.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1075,6 +1075,52 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:07</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>21.22</v>
+      </c>
+      <c r="D25" t="n">
+        <v>68</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Nuvens dispersas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BRASILIA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:08</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="D26" t="n">
+        <v>56</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Chuva leve</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implementado variaveis de ambiente para seguranca da API
</commit_message>
<xml_diff>
--- a/DadosClima/clima.xlsx
+++ b/DadosClima/clima.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1121,6 +1121,213 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:15</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>21.22</v>
+      </c>
+      <c r="D27" t="n">
+        <v>68</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nuvens dispersas</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PIAUI</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:16</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>26.52</v>
+      </c>
+      <c r="D28" t="n">
+        <v>56</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Nublado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:18</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="D29" t="n">
+        <v>68</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Nuvens dispersas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RECIFE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:18</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="D30" t="n">
+        <v>82</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Algumas nuvens</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OEIRAS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:18</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>27.28</v>
+      </c>
+      <c r="D31" t="n">
+        <v>42</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Nuvens dispersas</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TERESINA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>02/05/2026 21:19</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>28.84</v>
+      </c>
+      <c r="D32" t="n">
+        <v>74</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Algumas nuvens</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>02/05/2026 22:02</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>21.13</v>
+      </c>
+      <c r="D33" t="n">
+        <v>71</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Nuvens dispersas</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BAHIA</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>02/05/2026 22:03</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D34" t="n">
+        <v>77</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Nublado</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>OEIRAS</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>02/05/2026 22:03</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D35" t="n">
+        <v>47</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Nublado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>